<commit_message>
[hydgn/BHPSbP] smooth out trendline
</commit_message>
<xml_diff>
--- a/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
+++ b/InputData/hydgn/BHPSbP/BAU Hydrogen Production Shr by Pathway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lawrenceiu/Desktop/eps-us-3.4.7 working_D0228_T1015_woking/eps-us-3.4.7 HK working/InputData/hydgn/BHPSbP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdeng\Desktop\Dropbox_Free_Zone\EPS\Model Repos\China\Subnational\eps-hongkong\InputData\hydgn\BHPSbP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F08FA7E-EDB6-AD43-BED5-FB69CA584EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FBB3D58-9983-4018-8132-FD3F481801D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="25820" windowHeight="11980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2190" yWindow="1110" windowWidth="23595" windowHeight="12900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -107,7 +107,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -115,7 +115,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -123,24 +123,36 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -156,7 +168,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -166,10 +178,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
-    <cellStyle name="超連結" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -447,10 +461,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.796875" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -486,63 +500,63 @@
         <v>10</v>
       </c>
     </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+    </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="1" t="s">
-        <v>2</v>
+      <c r="A13" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" t="s">
-        <v>17</v>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="B15" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="B17" t="s">
-        <v>12</v>
+      <c r="B16" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="B18" t="s">
-        <v>13</v>
+      <c r="A18" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="B19" s="4" t="s">
-        <v>14</v>
+      <c r="A19">
+        <v>0.02</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20">
+        <v>0.76</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22">
-        <v>0.02</v>
-      </c>
-      <c r="B22" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23">
-        <v>0.76</v>
-      </c>
-      <c r="B23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24">
+      <c r="A21">
         <f>0.22</f>
         <v>0.22</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B21" t="s">
         <v>15</v>
       </c>
     </row>
@@ -550,7 +564,7 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B19" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B16" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>
@@ -563,9 +577,9 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AI6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.19921875" customWidth="1"/>
+    <col min="1" max="1" width="30.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35">
@@ -730,67 +744,79 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="5">
         <v>0.1</v>
       </c>
-      <c r="P2">
-        <v>0.1</v>
-      </c>
-      <c r="Q2">
-        <v>0.1</v>
-      </c>
-      <c r="R2">
-        <v>0.1</v>
-      </c>
-      <c r="S2">
-        <v>0.1</v>
-      </c>
-      <c r="T2">
+      <c r="P2" s="6">
+        <f>($T2-$O2)/COUNT($P$1:$T$1)+O2</f>
+        <v>0.12000000000000001</v>
+      </c>
+      <c r="Q2" s="6">
+        <f t="shared" ref="Q2:S3" si="1">($T2-$O2)/COUNT($P$1:$T$1)+P2</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="R2" s="6">
+        <f t="shared" si="1"/>
+        <v>0.16</v>
+      </c>
+      <c r="S2" s="6">
+        <f t="shared" si="1"/>
+        <v>0.18</v>
+      </c>
+      <c r="T2" s="5">
         <v>0.2</v>
       </c>
-      <c r="U2">
-        <v>0.2</v>
-      </c>
-      <c r="V2">
-        <v>0.2</v>
-      </c>
-      <c r="W2">
-        <v>0.2</v>
-      </c>
-      <c r="X2">
-        <v>0.2</v>
-      </c>
-      <c r="Y2">
+      <c r="U2" s="6">
+        <f>($Y2-$T2)/COUNT($U$1:$Y$1)+T2</f>
+        <v>0.26</v>
+      </c>
+      <c r="V2" s="6">
+        <f t="shared" ref="V2:X3" si="2">($Y2-$T2)/COUNT($U$1:$Y$1)+U2</f>
+        <v>0.32</v>
+      </c>
+      <c r="W2" s="6">
+        <f t="shared" si="2"/>
+        <v>0.38</v>
+      </c>
+      <c r="X2" s="6">
+        <f t="shared" si="2"/>
+        <v>0.44</v>
+      </c>
+      <c r="Y2" s="5">
         <v>0.5</v>
       </c>
-      <c r="Z2">
-        <v>0.5</v>
-      </c>
-      <c r="AA2">
-        <v>0.5</v>
-      </c>
-      <c r="AB2">
-        <v>0.5</v>
-      </c>
-      <c r="AC2">
-        <v>0.5</v>
-      </c>
-      <c r="AD2">
+      <c r="Z2" s="6">
+        <f>($AD2-$Y2)/COUNT($Z$1:$AD$1)+Y2</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="AA2" s="6">
+        <f t="shared" ref="AA2:AC3" si="3">($AD2-$Y2)/COUNT($Z$1:$AD$1)+Z2</f>
+        <v>0.62000000000000011</v>
+      </c>
+      <c r="AB2" s="6">
+        <f t="shared" si="3"/>
+        <v>0.68000000000000016</v>
+      </c>
+      <c r="AC2" s="6">
+        <f t="shared" si="3"/>
+        <v>0.74000000000000021</v>
+      </c>
+      <c r="AD2" s="5">
         <v>0.8</v>
       </c>
-      <c r="AE2">
+      <c r="AE2" s="5">
         <v>0.8</v>
       </c>
-      <c r="AF2">
+      <c r="AF2" s="5">
         <v>0.8</v>
       </c>
-      <c r="AG2">
+      <c r="AG2" s="5">
         <v>0.8</v>
       </c>
-      <c r="AH2">
+      <c r="AH2" s="5">
         <v>0.8</v>
       </c>
-      <c r="AI2">
+      <c r="AI2" s="5">
         <v>0.8</v>
       </c>
     </row>
@@ -802,114 +828,126 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <f t="shared" ref="C3:R6" si="1">$B3</f>
+        <f t="shared" ref="C3:N6" si="4">$B3</f>
         <v>1</v>
       </c>
       <c r="D3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="O3" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="P3" s="6">
+        <f>($T3-$O3)/COUNT($P$1:$T$1)+O3</f>
+        <v>0.88</v>
+      </c>
+      <c r="Q3" s="6">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="E3">
+        <v>0.86</v>
+      </c>
+      <c r="R3" s="6">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F3">
+        <v>0.84</v>
+      </c>
+      <c r="S3" s="6">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="O3">
-        <v>0.9</v>
-      </c>
-      <c r="P3">
-        <v>0.9</v>
-      </c>
-      <c r="Q3">
-        <v>0.9</v>
-      </c>
-      <c r="R3">
-        <v>0.9</v>
-      </c>
-      <c r="S3">
-        <v>0.9</v>
-      </c>
-      <c r="T3">
+        <v>0.82</v>
+      </c>
+      <c r="T3" s="5">
         <v>0.8</v>
       </c>
-      <c r="U3">
-        <v>0.8</v>
-      </c>
-      <c r="V3">
-        <v>0.8</v>
-      </c>
-      <c r="W3">
-        <v>0.8</v>
-      </c>
-      <c r="X3">
-        <v>0.8</v>
-      </c>
-      <c r="Y3">
+      <c r="U3" s="6">
+        <f>($Y3-$T3)/COUNT($U$1:$Y$1)+T3</f>
+        <v>0.74</v>
+      </c>
+      <c r="V3" s="6">
+        <f t="shared" si="2"/>
+        <v>0.67999999999999994</v>
+      </c>
+      <c r="W3" s="6">
+        <f t="shared" si="2"/>
+        <v>0.61999999999999988</v>
+      </c>
+      <c r="X3" s="6">
+        <f t="shared" si="2"/>
+        <v>0.55999999999999983</v>
+      </c>
+      <c r="Y3" s="5">
         <v>0.5</v>
       </c>
-      <c r="Z3">
-        <v>0.5</v>
-      </c>
-      <c r="AA3">
-        <v>0.5</v>
-      </c>
-      <c r="AB3">
-        <v>0.5</v>
-      </c>
-      <c r="AC3">
-        <v>0.5</v>
-      </c>
-      <c r="AD3">
+      <c r="Z3" s="6">
+        <f>($AD3-$Y3)/COUNT($Z$1:$AD$1)+Y3</f>
+        <v>0.44</v>
+      </c>
+      <c r="AA3" s="6">
+        <f t="shared" si="3"/>
+        <v>0.38</v>
+      </c>
+      <c r="AB3" s="6">
+        <f t="shared" si="3"/>
+        <v>0.32</v>
+      </c>
+      <c r="AC3" s="6">
+        <f t="shared" si="3"/>
+        <v>0.26</v>
+      </c>
+      <c r="AD3" s="5">
         <v>0.2</v>
       </c>
-      <c r="AE3">
+      <c r="AE3" s="5">
         <v>0.2</v>
       </c>
-      <c r="AF3">
+      <c r="AF3" s="5">
         <v>0.2</v>
       </c>
-      <c r="AG3">
+      <c r="AG3" s="5">
         <v>0.2</v>
       </c>
-      <c r="AH3">
+      <c r="AH3" s="5">
         <v>0.2</v>
       </c>
-      <c r="AI3">
+      <c r="AI3" s="5">
         <v>0.2</v>
       </c>
     </row>
@@ -921,7 +959,7 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="D4">
@@ -1061,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="D5">
@@ -1201,7 +1239,7 @@
         <v>0</v>
       </c>
       <c r="C6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="D6">
@@ -1340,15 +1378,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D257B2780BAD0A45A02FA065B9C6CC6A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="54b727ac31dab95898e9cf92f0402afe">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cb176f07-3112-4ee9-93fd-ae2cb5f3e433" xmlns:ns3="6b15a3a4-8173-42d6-9deb-398ec38eca4b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="42611c3eb46fef4c2b2610d1e51cc1b0" ns2:_="" ns3:_="">
     <xsd:import namespace="cb176f07-3112-4ee9-93fd-ae2cb5f3e433"/>
@@ -1597,15 +1626,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{859B11A2-12A3-4602-8E35-0801755A5680}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5D84DA1-2C59-4299-ABF0-55EA5DC3813C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1622,4 +1652,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{859B11A2-12A3-4602-8E35-0801755A5680}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>